<commit_message>
WB 2026-10-21: gráficas Dif vs Sin dif por proteína en hoja propia
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CP5rFdZnBGL53kJBCgrwYu
</commit_message>
<xml_diff>
--- a/resultados/wb/2026-10-21_cuantif_analisis.xlsx
+++ b/resultados/wb/2026-10-21_cuantif_analisis.xlsx
@@ -9,9 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="Analisis" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Hoja2" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Hoja3" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Hoja4" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Graficas" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Hoja2" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Hoja3" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Hoja4" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -57,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="106">
   <si>
     <t xml:space="preserve">Cuantificación WB queratinocitos diferenciados vs sin diferenciar — normalizado a 14-3-3ζ (canal 700)</t>
   </si>
@@ -189,6 +190,18 @@
   </si>
   <si>
     <t xml:space="preserve">n = 1–2 parejas por anticuerpo y sin saber si son réplicas biológicas o técnicas: no se calcula estadística.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datos de las gráficas: media de Diana / 14-3-3ζ por condición</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proteína</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K10 int no se grafica (sin banda). Valores de IVL Sin dif ≈ 0 (por debajo del límite de detección).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diana / 14-3-3ζ (media de parejas): Diferenciada vs Sin diferenciar</t>
   </si>
   <si>
     <t xml:space="preserve">Image Name</t>
@@ -527,7 +540,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -565,6 +578,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -626,7 +643,7 @@
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
       <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FFA5A5A5"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -666,7 +683,7 @@
                 </a:solidFill>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>log2 fold Dif / Sin dif (normalizado a 14-3-3ζ)</a:t>
+              <a:t>K14</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -688,17 +705,6 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Analisis!D47</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>log2 fold medio</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
           <c:spPr>
             <a:solidFill>
               <a:srgbClr val="4472c4"/>
@@ -708,7 +714,39 @@
             </a:ln>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a5a5a5"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
             <c:txPr>
               <a:bodyPr wrap="none"/>
               <a:lstStyle/>
@@ -735,62 +773,41 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Analisis!$A$48:$A$54</c:f>
+              <c:f>Analisis!$B$63:$C$63</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>K14</c:v>
+                  <c:v>Dif</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>K5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>K2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>K1</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>K10 ab</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>K10 int</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>IVL</c:v>
+                  <c:v>Sin dif</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Analisis!$D$48:$D$54</c:f>
+              <c:f>Analisis!$B$64:$C$64</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="7"/>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>-4.26920313871061</c:v>
+                  <c:v>0.781351813518135</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-5.55876891761755</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>-3.37084946591713</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>-5.52580128029055</c:v>
+                  <c:v>14.9042276980356</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:gapWidth val="150"/>
+        <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="18685560"/>
-        <c:axId val="75703172"/>
+        <c:axId val="61555573"/>
+        <c:axId val="29458412"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="18685560"/>
+        <c:axId val="61555573"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -822,7 +839,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75703172"/>
+        <c:crossAx val="29458412"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -830,22 +847,12 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75703172"/>
+        <c:axId val="29458412"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="6480">
-              <a:solidFill>
-                <a:srgbClr val="8b8b8b"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-          </c:spPr>
-        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -867,7 +874,7 @@
                     </a:solidFill>
                     <a:latin typeface="Calibri"/>
                   </a:rPr>
-                  <a:t>log2 (Dif / Sin dif)</a:t>
+                  <a:t>Diana / 14-3-3ζ</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -880,7 +887,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -906,7 +913,1427 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18685560"/>
+        <c:crossAx val="61555573"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>K5</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472c4"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a5a5a5"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analisis!$B$63:$C$63</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Dif</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sin dif</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analisis!$B$65:$C$65</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.0481871446320495</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.35736968345664</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="0"/>
+        <c:axId val="15801224"/>
+        <c:axId val="84542313"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="15801224"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="84542313"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="84542313"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Diana / 14-3-3ζ</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="15801224"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>K2</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472c4"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a5a5a5"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analisis!$B$63:$C$63</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Dif</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sin dif</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analisis!$B$66:$C$66</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.756681376875552</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>7.87589194699287</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="0"/>
+        <c:axId val="92119031"/>
+        <c:axId val="47967635"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="92119031"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="47967635"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="47967635"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Diana / 14-3-3ζ</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="92119031"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>K1</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472c4"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a5a5a5"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analisis!$B$63:$C$63</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Dif</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sin dif</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analisis!$B$67:$C$67</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.0215466270560104</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.02049689440994</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="0"/>
+        <c:axId val="1304784"/>
+        <c:axId val="83094413"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1304784"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="83094413"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="83094413"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Diana / 14-3-3ζ</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1304784"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>K10 ab</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472c4"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a5a5a5"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analisis!$B$63:$C$63</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Dif</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sin dif</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analisis!$B$68:$C$68</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>0.417193426042984</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.00175609756097561</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="0"/>
+        <c:axId val="3040582"/>
+        <c:axId val="69745708"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="3040582"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="69745708"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="69745708"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Diana / 14-3-3ζ</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="3040582"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>IVL</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472c4"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a5a5a5"/>
+              </a:solidFill>
+              <a:ln w="0">
+                <a:noFill/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="none"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:latin typeface="Arial"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:separator> </c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analisis!$B$63:$C$63</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Dif</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sin dif</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analisis!$B$69:$C$69</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>2.07213761438226</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0143258009528388</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="60"/>
+        <c:overlap val="0"/>
+        <c:axId val="86690692"/>
+        <c:axId val="52279174"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="86690692"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="52279174"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="52279174"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Diana / 14-3-3ζ</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="86690692"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -938,16 +2365,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>175680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>255960</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>7560</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>433440</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>38880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -955,12 +2382,162 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="9633600" y="6095880"/>
-        <a:ext cx="5759640" cy="2879640"/>
+        <a:off x="0" y="380880"/>
+        <a:ext cx="2879640" cy="2339640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>175680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>433800</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>38880</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="3669120" y="380880"/>
+        <a:ext cx="2879640" cy="2339640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>175680</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>433800</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>38880</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="7338240" y="380880"/>
+        <a:ext cx="2879640" cy="2339640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>433440</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>39240</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="3238560"/>
+        <a:ext cx="2879640" cy="2339640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>433800</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>39240</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 5"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="3669120" y="3238560"/>
+        <a:ext cx="2879640" cy="2339640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>433800</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>39240</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 6"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="7338240" y="3238560"/>
+        <a:ext cx="2879640" cy="2339640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -986,7 +2563,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Imagen 1" descr=""/>
+        <xdr:cNvPr id="6" name="Imagen 1" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1028,7 +2605,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen 1" descr=""/>
+        <xdr:cNvPr id="7" name="Imagen 1" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1065,7 +2642,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2" descr=""/>
+        <xdr:cNvPr id="8" name="Imagen 2" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1107,7 +2684,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Imagen 1" descr=""/>
+        <xdr:cNvPr id="9" name="Imagen 1" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1144,7 +2721,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Imagen 2" descr=""/>
+        <xdr:cNvPr id="10" name="Imagen 2" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1346,7 +2923,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -2781,6 +4358,105 @@
         <v>43</v>
       </c>
     </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B63" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B64" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A64,$D$6:$D$29,"Dif")</f>
+        <v>0.781351813518135</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A64,$D$6:$D$29,"Sin dif")</f>
+        <v>14.9042276980356</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B65" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A65,$D$6:$D$29,"Dif")</f>
+        <v>0.0481871446320495</v>
+      </c>
+      <c r="C65" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A65,$D$6:$D$29,"Sin dif")</f>
+        <v>2.35736968345664</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B66" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A66,$D$6:$D$29,"Dif")</f>
+        <v>0.756681376875552</v>
+      </c>
+      <c r="C66" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A66,$D$6:$D$29,"Sin dif")</f>
+        <v>7.87589194699287</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B67" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A67,$D$6:$D$29,"Dif")</f>
+        <v>0.0215466270560104</v>
+      </c>
+      <c r="C67" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A67,$D$6:$D$29,"Sin dif")</f>
+        <v>1.02049689440994</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A68,$D$6:$D$29,"Dif")</f>
+        <v>0.417193426042984</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A68,$D$6:$D$29,"Sin dif")</f>
+        <v>0.00175609756097561</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B69" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A69,$D$6:$D$29,"Dif")</f>
+        <v>2.07213761438226</v>
+      </c>
+      <c r="C69" s="7" t="n">
+        <f aca="false">AVERAGEIFS($I$6:$I$29,$B$6:$B$29,$A69,$D$6:$D$29,"Sin dif")</f>
+        <v>0.0143258009528388</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2789,8 +4465,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2800,10 +4475,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -2837,33 +4518,52 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:H48"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2871,7 +4571,7 @@
         <v>3461</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C2" s="0" t="n">
         <v>1</v>
@@ -2886,10 +4586,10 @@
         <v>3072</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2897,7 +4597,7 @@
         <v>3461</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C3" s="0" t="n">
         <v>2</v>
@@ -2912,10 +4612,10 @@
         <v>3072</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2923,7 +4623,7 @@
         <v>3461</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C4" s="0" t="n">
         <v>3</v>
@@ -2938,10 +4638,10 @@
         <v>3072</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2949,7 +4649,7 @@
         <v>3461</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C5" s="0" t="n">
         <v>4</v>
@@ -2964,10 +4664,10 @@
         <v>2310</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2975,7 +4675,7 @@
         <v>3461</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C6" s="0" t="n">
         <v>5</v>
@@ -2990,10 +4690,10 @@
         <v>3072</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3001,7 +4701,7 @@
         <v>3461</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C7" s="0" t="n">
         <v>6</v>
@@ -3016,10 +4716,10 @@
         <v>2250</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,7 +4727,7 @@
         <v>3461</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C8" s="0" t="n">
         <v>7</v>
@@ -3042,10 +4742,10 @@
         <v>3384</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3053,7 +4753,7 @@
         <v>3461</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C9" s="0" t="n">
         <v>8</v>
@@ -3068,10 +4768,10 @@
         <v>2250</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3079,7 +4779,7 @@
         <v>3461</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C10" s="0" t="n">
         <v>9</v>
@@ -3094,10 +4794,10 @@
         <v>2560</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3105,7 +4805,7 @@
         <v>3461</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C11" s="0" t="n">
         <v>10</v>
@@ -3120,10 +4820,10 @@
         <v>2560</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3131,7 +4831,7 @@
         <v>3461</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C12" s="0" t="n">
         <v>11</v>
@@ -3146,10 +4846,10 @@
         <v>2656</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3157,7 +4857,7 @@
         <v>3461</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C13" s="0" t="n">
         <v>12</v>
@@ -3172,10 +4872,10 @@
         <v>2560</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3183,7 +4883,7 @@
         <v>3461</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C14" s="0" t="n">
         <v>13</v>
@@ -3198,10 +4898,10 @@
         <v>2560</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3209,7 +4909,7 @@
         <v>3461</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" s="0" t="n">
         <v>14</v>
@@ -3224,10 +4924,10 @@
         <v>2560</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3235,7 +4935,7 @@
         <v>3461</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C16" s="0" t="n">
         <v>15</v>
@@ -3250,10 +4950,10 @@
         <v>2560</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3261,7 +4961,7 @@
         <v>3461</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C17" s="0" t="n">
         <v>16</v>
@@ -3276,10 +4976,10 @@
         <v>2560</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3287,7 +4987,7 @@
         <v>3461</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C18" s="0" t="n">
         <v>17</v>
@@ -3302,10 +5002,10 @@
         <v>3003</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3313,7 +5013,7 @@
         <v>3461</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C19" s="0" t="n">
         <v>18</v>
@@ -3328,10 +5028,10 @@
         <v>2560</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3339,7 +5039,7 @@
         <v>3461</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C20" s="0" t="n">
         <v>19</v>
@@ -3354,10 +5054,10 @@
         <v>2560</v>
       </c>
       <c r="G20" s="0" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H20" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3365,7 +5065,7 @@
         <v>3461</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C21" s="0" t="n">
         <v>20</v>
@@ -3380,10 +5080,10 @@
         <v>2560</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3391,7 +5091,7 @@
         <v>3461</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C22" s="0" t="n">
         <v>21</v>
@@ -3406,10 +5106,10 @@
         <v>2560</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3417,7 +5117,7 @@
         <v>3461</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C23" s="0" t="n">
         <v>22</v>
@@ -3432,10 +5132,10 @@
         <v>2560</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3443,7 +5143,7 @@
         <v>3461</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C24" s="0" t="n">
         <v>23</v>
@@ -3458,10 +5158,10 @@
         <v>2560</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3469,7 +5169,7 @@
         <v>3461</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C25" s="0" t="n">
         <v>24</v>
@@ -3484,10 +5184,10 @@
         <v>2560</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3495,7 +5195,7 @@
         <v>3461</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C26" s="0" t="n">
         <v>25</v>
@@ -3510,10 +5210,10 @@
         <v>2844</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3521,7 +5221,7 @@
         <v>3461</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C27" s="0" t="n">
         <v>26</v>
@@ -3536,10 +5236,10 @@
         <v>2844</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3547,7 +5247,7 @@
         <v>3461</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C28" s="0" t="n">
         <v>27</v>
@@ -3562,10 +5262,10 @@
         <v>2844</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3573,7 +5273,7 @@
         <v>3461</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C29" s="0" t="n">
         <v>28</v>
@@ -3588,10 +5288,10 @@
         <v>2844</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3599,7 +5299,7 @@
         <v>3461</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C30" s="0" t="n">
         <v>29</v>
@@ -3614,10 +5314,10 @@
         <v>1975</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3625,7 +5325,7 @@
         <v>3461</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C31" s="0" t="n">
         <v>30</v>
@@ -3640,10 +5340,10 @@
         <v>2844</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3651,7 +5351,7 @@
         <v>3461</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C32" s="0" t="n">
         <v>31</v>
@@ -3666,10 +5366,10 @@
         <v>2844</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3677,7 +5377,7 @@
         <v>3461</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C33" s="0" t="n">
         <v>32</v>
@@ -3692,10 +5392,10 @@
         <v>2844</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3703,7 +5403,7 @@
         <v>3461</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C34" s="0" t="n">
         <v>33</v>
@@ -3718,10 +5418,10 @@
         <v>2844</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3729,7 +5429,7 @@
         <v>3461</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C35" s="0" t="n">
         <v>34</v>
@@ -3744,10 +5444,10 @@
         <v>2975</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3755,7 +5455,7 @@
         <v>3461</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C36" s="0" t="n">
         <v>35</v>
@@ -3770,10 +5470,10 @@
         <v>2844</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3781,7 +5481,7 @@
         <v>3461</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C37" s="0" t="n">
         <v>36</v>
@@ -3796,10 +5496,10 @@
         <v>2844</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3807,7 +5507,7 @@
         <v>3461</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C38" s="0" t="n">
         <v>37</v>
@@ -3822,10 +5522,10 @@
         <v>2844</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3833,7 +5533,7 @@
         <v>3461</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C39" s="0" t="n">
         <v>38</v>
@@ -3848,10 +5548,10 @@
         <v>2844</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H39" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3859,7 +5559,7 @@
         <v>3461</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C40" s="0" t="n">
         <v>39</v>
@@ -3874,10 +5574,10 @@
         <v>2844</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3885,7 +5585,7 @@
         <v>3461</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C41" s="0" t="n">
         <v>40</v>
@@ -3900,10 +5600,10 @@
         <v>2844</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3911,7 +5611,7 @@
         <v>3461</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C42" s="0" t="n">
         <v>41</v>
@@ -3926,10 +5626,10 @@
         <v>2844</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H42" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3937,7 +5637,7 @@
         <v>3461</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C43" s="0" t="n">
         <v>42</v>
@@ -3952,10 +5652,10 @@
         <v>2844</v>
       </c>
       <c r="G43" s="0" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H43" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3963,7 +5663,7 @@
         <v>3461</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C44" s="0" t="n">
         <v>43</v>
@@ -3978,10 +5678,10 @@
         <v>2844</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3989,7 +5689,7 @@
         <v>3461</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C45" s="0" t="n">
         <v>44</v>
@@ -4004,10 +5704,10 @@
         <v>2844</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4015,25 +5715,25 @@
         <v>3461</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C46" s="0" t="n">
         <v>45</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F46" s="0" t="n">
         <v>2844</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="H46" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4041,13 +5741,13 @@
         <v>3461</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C47" s="0" t="n">
         <v>46</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E47" s="0" t="n">
         <v>570</v>
@@ -4056,10 +5756,10 @@
         <v>2844</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4067,13 +5767,13 @@
         <v>3461</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C48" s="0" t="n">
         <v>47</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E48" s="0" t="n">
         <v>406</v>
@@ -4082,10 +5782,10 @@
         <v>2844</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WB 2026-10-21: comparación ARNm (qPCR MD2) vs proteína e incorpora Hoja1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CP5rFdZnBGL53kJBCgrwYu
</commit_message>
<xml_diff>
--- a/resultados/wb/2026-10-21_cuantif_analisis.xlsx
+++ b/resultados/wb/2026-10-21_cuantif_analisis.xlsx
@@ -10,9 +10,11 @@
   <sheets>
     <sheet name="Analisis" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Graficas" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Hoja2" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Hoja3" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Hoja4" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="ARNm vs proteina" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Hoja1" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Hoja2" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Hoja3" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Hoja4" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -58,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="151">
   <si>
     <t xml:space="preserve">Cuantificación WB queratinocitos diferenciados vs sin diferenciar — normalizado a 14-3-3ζ (canal 700)</t>
   </si>
@@ -202,6 +204,141 @@
   </si>
   <si>
     <t xml:space="preserve">Diana / 14-3-3ζ (media de parejas): Diferenciada vs Sin diferenciar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MD2: ARNm (qPCR, 7 d vs 0 d) frente a proteína (WB, Dif vs Sin dif)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNm: RQ 2^-ΔΔCt con YWHAZ, de qPCR_analisis_MD2_MD3.xlsx (hoja Resumen; azul = copiado de ese archivo). Proteína: fold de la hoja Analisis (fórmulas).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: WB «Sin dif» = KerCT WT / 0 días y «Dif» = KerCT MD2 7 días (Hoja1). Fold &gt; 1 = más en diferenciado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K10 e IVL: la barra de proteína es un mínimo (en Sin dif no hay banda).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNm MD2 rep 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNm MD2 rep 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNm 7d/0d (media)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proteína Dif/Sin dif (norm. 14-3-3ζ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proteína Dif/Sin dif (señal bruta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Proteína es un mínimo?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Mismo sentido ARNm y proteína?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comentario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KRT1 / K1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNm casi ausente a 0 d (Ct ≈ 32) pero el WB da banda fuerte en Sin dif: la banda probablemente no es K1 (reacción cruzada).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KRT2 / K2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARNm muy bajo en ambas (Ct ≈ 30–31): la banda fuerte en Sin dif del WB es sospechosa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KRT10 / K10 (ab)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí (≥)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concuerdan: K10 solo detectable en Dif. El valor de proteína es un mínimo (Sin dif bajo el límite de detección).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KRT14 / K14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concuerdan (bajan). La proteína sin normalizar (~0,3) se parece mucho al ARNm (~0,4); normalizada a 14-3-3ζ se exagera.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concuerdan: IVL solo detectable en Dif. Valor de proteína = mínimo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KRT5 / K5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no medido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sin dato de ARNm en MD2 (en Medio 3D sí). Proteína baja con la diferenciación, como se espera.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La media de ARNm es geométrica entre MD2 rep 1 y rep 2. En proteína: media geométrica de las parejas del WB.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• K14, K10 e IVL: ARNm y proteína van en el mismo sentido (K14 baja; K10 e IVL suben, y en proteína solo aparecen en diferenciado).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• K1 y K2: discrepancia total. El ARNm sube con la diferenciación (K1 ~56×, K2 ~2,4×) pero el WB da más señal en Sin dif, incluso sin normalizar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   A 0 d el ARNm de KRT1 y KRT2 está casi en el límite (Ct 30–32), así que una banda fuerte en Sin dif no es creíble: revisar especificidad del anticuerpo / altura de la banda (K1 ~67 kDa, K2 ~65 kDa; K5 ~58 kDa, K14 ~50 kDa).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• 14-3-3ζ (YWHAZ): el ARNm apenas cambia (Ct 16,4 a 0 d frente a 16,0 a 7 d en MD2, ~1,3×), pero la proteína sale 4–8× más alta en Dif con la misma carga teórica (30 µg).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Eso apunta a carga desigual / cuantificación de proteína, más que a un cambio real de 14-3-3ζ. Con señal sin normalizar, K14 (0,3×) coincide con el ARNm (0,4×).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Magnitudes: no son comparables 1:1 (el WB satura y tiene menos rango dinámico que la qPCR); lo comparable es el sentido del cambio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentración </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ul para 30ng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ul agente reductor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ul tampón carga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ul H2O</t>
+  </si>
+  <si>
+    <t xml:space="preserve">volumen final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cuántas?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KerCT WT </t>
+  </si>
+  <si>
+    <t xml:space="preserve">KerCT MD2 7 días</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1:5000 el de K10 abcam al final</t>
   </si>
   <si>
     <t xml:space="preserve">Image Name</t>
@@ -382,11 +519,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00"/>
+    <numFmt numFmtId="168" formatCode="0.0#"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -540,7 +678,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -582,6 +720,34 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -641,7 +807,7 @@
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FFED7D31"/>
       <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FFA5A5A5"/>
       <rgbColor rgb="FF003366"/>
@@ -803,11 +969,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="61555573"/>
-        <c:axId val="29458412"/>
+        <c:axId val="98657918"/>
+        <c:axId val="12218026"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="61555573"/>
+        <c:axId val="98657918"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -839,7 +1005,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29458412"/>
+        <c:crossAx val="12218026"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -847,7 +1013,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="29458412"/>
+        <c:axId val="12218026"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -913,7 +1079,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61555573"/>
+        <c:crossAx val="98657918"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1087,11 +1253,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="15801224"/>
-        <c:axId val="84542313"/>
+        <c:axId val="61948173"/>
+        <c:axId val="86907954"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="15801224"/>
+        <c:axId val="61948173"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1123,7 +1289,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84542313"/>
+        <c:crossAx val="86907954"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1131,7 +1297,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84542313"/>
+        <c:axId val="86907954"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1197,7 +1363,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15801224"/>
+        <c:crossAx val="61948173"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1371,11 +1537,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="92119031"/>
-        <c:axId val="47967635"/>
+        <c:axId val="83474198"/>
+        <c:axId val="20579682"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="92119031"/>
+        <c:axId val="83474198"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1407,7 +1573,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47967635"/>
+        <c:crossAx val="20579682"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1415,7 +1581,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47967635"/>
+        <c:axId val="20579682"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1481,7 +1647,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92119031"/>
+        <c:crossAx val="83474198"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1655,11 +1821,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="1304784"/>
-        <c:axId val="83094413"/>
+        <c:axId val="84993984"/>
+        <c:axId val="63907181"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1304784"/>
+        <c:axId val="84993984"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1691,7 +1857,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="83094413"/>
+        <c:crossAx val="63907181"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1699,7 +1865,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="83094413"/>
+        <c:axId val="63907181"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1765,7 +1931,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1304784"/>
+        <c:crossAx val="84993984"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1939,11 +2105,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="3040582"/>
-        <c:axId val="69745708"/>
+        <c:axId val="14693973"/>
+        <c:axId val="5077888"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="3040582"/>
+        <c:axId val="14693973"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1975,7 +2141,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69745708"/>
+        <c:crossAx val="5077888"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1983,7 +2149,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="69745708"/>
+        <c:axId val="5077888"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2049,7 +2215,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3040582"/>
+        <c:crossAx val="14693973"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2223,11 +2389,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="86690692"/>
-        <c:axId val="52279174"/>
+        <c:axId val="76649506"/>
+        <c:axId val="60497147"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86690692"/>
+        <c:axId val="76649506"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2259,7 +2425,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52279174"/>
+        <c:crossAx val="60497147"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2267,7 +2433,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52279174"/>
+        <c:axId val="60497147"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2333,7 +2499,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86690692"/>
+        <c:crossAx val="76649506"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2344,6 +2510,520 @@
         </a:ln>
       </c:spPr>
     </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Fold diferenciado vs sin diferenciar (MD2)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ARNm vs proteina'!D5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>ARNm 7d/0d (media)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4472c4"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="4472c4"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ARNm vs proteina'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>KRT1 / K1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>KRT2 / K2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>KRT10 / K10 (ab)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>KRT14 / K14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>IVL</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ARNm vs proteina'!$D$6:$D$10</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>54.5001756877902</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.35716142849827</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>22.7717358143818</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.381200734521853</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>169.772270138559</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ARNm vs proteina'!F5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Proteína Dif/Sin dif (señal bruta)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="a5a5a5"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="a5a5a5"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ARNm vs proteina'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>KRT1 / K1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>KRT2 / K2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>KRT10 / K10 (ab)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>KRT14 / K14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>IVL</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ARNm vs proteina'!$F$6:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0.145156707728777</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.580735883742917</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.289231726052959</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>143.013985330107</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'ARNm vs proteina'!E5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Proteína Dif/Sin dif (norm. 14-3-3ζ)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="ed7d31"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:solidFill>
+                <a:srgbClr val="ed7d31"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'ARNm vs proteina'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>KRT1 / K1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>KRT2 / K2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>KRT10 / K10 (ab)</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>KRT14 / K14</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>IVL</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'ARNm vs proteina'!$E$6:$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0.0217054135376413</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0966658779933537</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.55246523388116</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.0518611087805558</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>30.7516299425454</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="54902850"/>
+        <c:axId val="62689967"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="54902850"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="62689967"/>
+        <c:crossesAt val="1"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="62689967"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6480">
+              <a:solidFill>
+                <a:srgbClr val="8b8b8b"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Fold (escala log)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.0#" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6480">
+            <a:solidFill>
+              <a:srgbClr val="8b8b8b"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="54902850"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
   </c:chart>
@@ -2550,6 +3230,83 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>364320</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>54720</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="12170880" y="762120"/>
+        <a:ext cx="6479640" cy="3239640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>409680</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>171360</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="1143000"/>
+          <a:ext cx="7629120" cy="3981240"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
@@ -2563,7 +3320,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Imagen 1" descr=""/>
+        <xdr:cNvPr id="8" name="Imagen 1" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2588,7 +3345,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2605,7 +3362,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Imagen 1" descr=""/>
+        <xdr:cNvPr id="9" name="Imagen 1" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2642,7 +3399,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Imagen 2" descr=""/>
+        <xdr:cNvPr id="10" name="Imagen 2" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2667,7 +3424,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2684,7 +3441,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Imagen 1" descr=""/>
+        <xdr:cNvPr id="11" name="Imagen 1" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -2721,7 +3478,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Imagen 2" descr=""/>
+        <xdr:cNvPr id="12" name="Imagen 2" descr=""/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -4499,11 +5256,299 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K4" s="2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>68.645</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>43.27</v>
+      </c>
+      <c r="D6" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(B6),LOG(C6))</f>
+        <v>54.5001756877902</v>
+      </c>
+      <c r="E6" s="14" t="n">
+        <f aca="false">Analisis!C51</f>
+        <v>0.0217054135376413</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(Analisis!G37),LOG(Analisis!G38))</f>
+        <v>0.145156707728777</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H6" s="12" t="str">
+        <f aca="false">IF(SIGN(LOG(D6))=SIGN(LOG(E6)),"Sí","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>2.486</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>2.235</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(B7),LOG(C7))</f>
+        <v>2.35716142849827</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <f aca="false">Analisis!C50</f>
+        <v>0.0966658779933537</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(Analisis!G39),LOG(Analisis!G40))</f>
+        <v>0.580735883742917</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="12" t="str">
+        <f aca="false">IF(SIGN(LOG(D7))=SIGN(LOG(E7)),"Sí","NO")</f>
+        <v>NO</v>
+      </c>
+      <c r="I7" s="12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>24.548</v>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>21.124</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(B8),LOG(C8))</f>
+        <v>22.7717358143818</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <f aca="false">(Analisis!I16/(Analisis!$G$3/Analisis!H17))</f>
+        <v>8.55246523388116</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <f aca="false">(Analisis!F16/Analisis!$G$3)</f>
+        <v>33</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="H8" s="12" t="str">
+        <f aca="false">IF(SIGN(LOG(D8))=SIGN(LOG(E8)),"Sí","NO")</f>
+        <v>Sí</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>0.351</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(B9),LOG(C9))</f>
+        <v>0.381200734521853</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <f aca="false">Analisis!C48</f>
+        <v>0.0518611087805558</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(Analisis!G33),LOG(Analisis!G34))</f>
+        <v>0.289231726052959</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="12" t="str">
+        <f aca="false">IF(SIGN(LOG(D9))=SIGN(LOG(E9)),"Sí","NO")</f>
+        <v>Sí</v>
+      </c>
+      <c r="I9" s="12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>177.766</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>162.138</v>
+      </c>
+      <c r="D10" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(B10),LOG(C10))</f>
+        <v>169.772270138559</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(Analisis!I26/(Analisis!$G$3/Analisis!H27)),LOG(Analisis!I28/(Analisis!$G$3/Analisis!H29)))</f>
+        <v>30.7516299425454</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <f aca="false">10^AVERAGE(LOG(Analisis!F26/Analisis!$G$3),LOG(Analisis!F28/Analisis!$G$3))</f>
+        <v>143.013985330107</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="H10" s="12" t="str">
+        <f aca="false">IF(SIGN(LOG(D10))=SIGN(LOG(E10)),"Sí","NO")</f>
+        <v>Sí</v>
+      </c>
+      <c r="I10" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="9" t="n">
+        <f aca="false">Analisis!C49</f>
+        <v>0.0212150381381759</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <f aca="false">10^AVERAGE(LOG(Analisis!G35),LOG(Analisis!G36))</f>
+        <v>0.0955483658154862</v>
+      </c>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
@@ -4514,6 +5559,120 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.66"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="H1" s="17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>4.085</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <f aca="false">30/B2</f>
+        <v>7.34394124847001</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <f aca="false">G2/10</f>
+        <v>1.5</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <f aca="false">G2/4</f>
+        <v>3.75</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <f aca="false">G2-C2-E2</f>
+        <v>3.90605875152999</v>
+      </c>
+      <c r="G2" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="H2" s="0" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <f aca="false">30/B3</f>
+        <v>2.17391304347826</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <f aca="false">G3/10</f>
+        <v>1.5</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <f aca="false">G3/4</f>
+        <v>3.75</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <f aca="false">G3-C3-E3</f>
+        <v>9.07608695652174</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="H3" s="0" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G38" s="0" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4532,7 +5691,26 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -4542,28 +5720,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>49</v>
+        <v>94</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>50</v>
+        <v>95</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>52</v>
+        <v>97</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>55</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4571,7 +5749,7 @@
         <v>3461</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C2" s="0" t="n">
         <v>1</v>
@@ -4586,10 +5764,10 @@
         <v>3072</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4597,7 +5775,7 @@
         <v>3461</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C3" s="0" t="n">
         <v>2</v>
@@ -4612,10 +5790,10 @@
         <v>3072</v>
       </c>
       <c r="G3" s="0" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="H3" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4623,7 +5801,7 @@
         <v>3461</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C4" s="0" t="n">
         <v>3</v>
@@ -4638,10 +5816,10 @@
         <v>3072</v>
       </c>
       <c r="G4" s="0" t="s">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="H4" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4649,7 +5827,7 @@
         <v>3461</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C5" s="0" t="n">
         <v>4</v>
@@ -4664,10 +5842,10 @@
         <v>2310</v>
       </c>
       <c r="G5" s="0" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4675,7 +5853,7 @@
         <v>3461</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C6" s="0" t="n">
         <v>5</v>
@@ -4690,10 +5868,10 @@
         <v>3072</v>
       </c>
       <c r="G6" s="0" t="s">
-        <v>61</v>
+        <v>106</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4701,7 +5879,7 @@
         <v>3461</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C7" s="0" t="n">
         <v>6</v>
@@ -4716,10 +5894,10 @@
         <v>2250</v>
       </c>
       <c r="G7" s="0" t="s">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4727,7 +5905,7 @@
         <v>3461</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C8" s="0" t="n">
         <v>7</v>
@@ -4742,10 +5920,10 @@
         <v>3384</v>
       </c>
       <c r="G8" s="0" t="s">
-        <v>58</v>
+        <v>103</v>
       </c>
       <c r="H8" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4753,7 +5931,7 @@
         <v>3461</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C9" s="0" t="n">
         <v>8</v>
@@ -4768,10 +5946,10 @@
         <v>2250</v>
       </c>
       <c r="G9" s="0" t="s">
-        <v>62</v>
+        <v>107</v>
       </c>
       <c r="H9" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4779,7 +5957,7 @@
         <v>3461</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C10" s="0" t="n">
         <v>9</v>
@@ -4794,10 +5972,10 @@
         <v>2560</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>63</v>
+        <v>108</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4805,7 +5983,7 @@
         <v>3461</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C11" s="0" t="n">
         <v>10</v>
@@ -4820,10 +5998,10 @@
         <v>2560</v>
       </c>
       <c r="G11" s="0" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
       <c r="H11" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4831,7 +6009,7 @@
         <v>3461</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C12" s="0" t="n">
         <v>11</v>
@@ -4846,10 +6024,10 @@
         <v>2656</v>
       </c>
       <c r="G12" s="0" t="s">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="H12" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4857,7 +6035,7 @@
         <v>3461</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C13" s="0" t="n">
         <v>12</v>
@@ -4872,10 +6050,10 @@
         <v>2560</v>
       </c>
       <c r="G13" s="0" t="s">
-        <v>66</v>
+        <v>111</v>
       </c>
       <c r="H13" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4883,7 +6061,7 @@
         <v>3461</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C14" s="0" t="n">
         <v>13</v>
@@ -4898,10 +6076,10 @@
         <v>2560</v>
       </c>
       <c r="G14" s="0" t="s">
-        <v>67</v>
+        <v>112</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4909,7 +6087,7 @@
         <v>3461</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C15" s="0" t="n">
         <v>14</v>
@@ -4924,10 +6102,10 @@
         <v>2560</v>
       </c>
       <c r="G15" s="0" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4935,7 +6113,7 @@
         <v>3461</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C16" s="0" t="n">
         <v>15</v>
@@ -4950,10 +6128,10 @@
         <v>2560</v>
       </c>
       <c r="G16" s="0" t="s">
-        <v>69</v>
+        <v>114</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4961,7 +6139,7 @@
         <v>3461</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C17" s="0" t="n">
         <v>16</v>
@@ -4976,10 +6154,10 @@
         <v>2560</v>
       </c>
       <c r="G17" s="0" t="s">
-        <v>70</v>
+        <v>115</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4987,7 +6165,7 @@
         <v>3461</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C18" s="0" t="n">
         <v>17</v>
@@ -5002,10 +6180,10 @@
         <v>3003</v>
       </c>
       <c r="G18" s="0" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
       <c r="H18" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5013,7 +6191,7 @@
         <v>3461</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C19" s="0" t="n">
         <v>18</v>
@@ -5028,10 +6206,10 @@
         <v>2560</v>
       </c>
       <c r="G19" s="0" t="s">
-        <v>71</v>
+        <v>116</v>
       </c>
       <c r="H19" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5039,7 +6217,7 @@
         <v>3461</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C20" s="0" t="n">
         <v>19</v>
@@ -5054,10 +6232,10 @@
         <v>2560</v>
       </c>
       <c r="G20" s="0" t="s">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="H20" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5065,7 +6243,7 @@
         <v>3461</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C21" s="0" t="n">
         <v>20</v>
@@ -5080,10 +6258,10 @@
         <v>2560</v>
       </c>
       <c r="G21" s="0" t="s">
-        <v>73</v>
+        <v>118</v>
       </c>
       <c r="H21" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5091,7 +6269,7 @@
         <v>3461</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C22" s="0" t="n">
         <v>21</v>
@@ -5106,10 +6284,10 @@
         <v>2560</v>
       </c>
       <c r="G22" s="0" t="s">
-        <v>74</v>
+        <v>119</v>
       </c>
       <c r="H22" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5117,7 +6295,7 @@
         <v>3461</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C23" s="0" t="n">
         <v>22</v>
@@ -5132,10 +6310,10 @@
         <v>2560</v>
       </c>
       <c r="G23" s="0" t="s">
-        <v>75</v>
+        <v>120</v>
       </c>
       <c r="H23" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5143,7 +6321,7 @@
         <v>3461</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C24" s="0" t="n">
         <v>23</v>
@@ -5158,10 +6336,10 @@
         <v>2560</v>
       </c>
       <c r="G24" s="0" t="s">
-        <v>76</v>
+        <v>121</v>
       </c>
       <c r="H24" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5169,7 +6347,7 @@
         <v>3461</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>56</v>
+        <v>101</v>
       </c>
       <c r="C25" s="0" t="n">
         <v>24</v>
@@ -5184,10 +6362,10 @@
         <v>2560</v>
       </c>
       <c r="G25" s="0" t="s">
-        <v>77</v>
+        <v>122</v>
       </c>
       <c r="H25" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5195,7 +6373,7 @@
         <v>3461</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C26" s="0" t="n">
         <v>25</v>
@@ -5210,10 +6388,10 @@
         <v>2844</v>
       </c>
       <c r="G26" s="0" t="s">
-        <v>79</v>
+        <v>124</v>
       </c>
       <c r="H26" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5221,7 +6399,7 @@
         <v>3461</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C27" s="0" t="n">
         <v>26</v>
@@ -5236,10 +6414,10 @@
         <v>2844</v>
       </c>
       <c r="G27" s="0" t="s">
-        <v>80</v>
+        <v>125</v>
       </c>
       <c r="H27" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5247,7 +6425,7 @@
         <v>3461</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C28" s="0" t="n">
         <v>27</v>
@@ -5262,10 +6440,10 @@
         <v>2844</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>81</v>
+        <v>126</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5273,7 +6451,7 @@
         <v>3461</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C29" s="0" t="n">
         <v>28</v>
@@ -5288,10 +6466,10 @@
         <v>2844</v>
       </c>
       <c r="G29" s="0" t="s">
-        <v>82</v>
+        <v>127</v>
       </c>
       <c r="H29" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5299,7 +6477,7 @@
         <v>3461</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C30" s="0" t="n">
         <v>29</v>
@@ -5314,10 +6492,10 @@
         <v>1975</v>
       </c>
       <c r="G30" s="0" t="s">
-        <v>83</v>
+        <v>128</v>
       </c>
       <c r="H30" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5325,7 +6503,7 @@
         <v>3461</v>
       </c>
       <c r="B31" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C31" s="0" t="n">
         <v>30</v>
@@ -5340,10 +6518,10 @@
         <v>2844</v>
       </c>
       <c r="G31" s="0" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="H31" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5351,7 +6529,7 @@
         <v>3461</v>
       </c>
       <c r="B32" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C32" s="0" t="n">
         <v>31</v>
@@ -5366,10 +6544,10 @@
         <v>2844</v>
       </c>
       <c r="G32" s="0" t="s">
-        <v>85</v>
+        <v>130</v>
       </c>
       <c r="H32" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5377,7 +6555,7 @@
         <v>3461</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C33" s="0" t="n">
         <v>32</v>
@@ -5392,10 +6570,10 @@
         <v>2844</v>
       </c>
       <c r="G33" s="0" t="s">
-        <v>86</v>
+        <v>131</v>
       </c>
       <c r="H33" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5403,7 +6581,7 @@
         <v>3461</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C34" s="0" t="n">
         <v>33</v>
@@ -5418,10 +6596,10 @@
         <v>2844</v>
       </c>
       <c r="G34" s="0" t="s">
-        <v>87</v>
+        <v>132</v>
       </c>
       <c r="H34" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5429,7 +6607,7 @@
         <v>3461</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C35" s="0" t="n">
         <v>34</v>
@@ -5444,10 +6622,10 @@
         <v>2975</v>
       </c>
       <c r="G35" s="0" t="s">
-        <v>88</v>
+        <v>133</v>
       </c>
       <c r="H35" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5455,7 +6633,7 @@
         <v>3461</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C36" s="0" t="n">
         <v>35</v>
@@ -5470,10 +6648,10 @@
         <v>2844</v>
       </c>
       <c r="G36" s="0" t="s">
-        <v>89</v>
+        <v>134</v>
       </c>
       <c r="H36" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5481,7 +6659,7 @@
         <v>3461</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C37" s="0" t="n">
         <v>36</v>
@@ -5496,10 +6674,10 @@
         <v>2844</v>
       </c>
       <c r="G37" s="0" t="s">
-        <v>90</v>
+        <v>135</v>
       </c>
       <c r="H37" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5507,7 +6685,7 @@
         <v>3461</v>
       </c>
       <c r="B38" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C38" s="0" t="n">
         <v>37</v>
@@ -5522,10 +6700,10 @@
         <v>2844</v>
       </c>
       <c r="G38" s="0" t="s">
-        <v>91</v>
+        <v>136</v>
       </c>
       <c r="H38" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5533,7 +6711,7 @@
         <v>3461</v>
       </c>
       <c r="B39" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C39" s="0" t="n">
         <v>38</v>
@@ -5548,10 +6726,10 @@
         <v>2844</v>
       </c>
       <c r="G39" s="0" t="s">
-        <v>92</v>
+        <v>137</v>
       </c>
       <c r="H39" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5559,7 +6737,7 @@
         <v>3461</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C40" s="0" t="n">
         <v>39</v>
@@ -5574,10 +6752,10 @@
         <v>2844</v>
       </c>
       <c r="G40" s="0" t="s">
-        <v>93</v>
+        <v>138</v>
       </c>
       <c r="H40" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5585,7 +6763,7 @@
         <v>3461</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C41" s="0" t="n">
         <v>40</v>
@@ -5600,10 +6778,10 @@
         <v>2844</v>
       </c>
       <c r="G41" s="0" t="s">
-        <v>94</v>
+        <v>139</v>
       </c>
       <c r="H41" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5611,7 +6789,7 @@
         <v>3461</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C42" s="0" t="n">
         <v>41</v>
@@ -5626,10 +6804,10 @@
         <v>2844</v>
       </c>
       <c r="G42" s="0" t="s">
-        <v>95</v>
+        <v>140</v>
       </c>
       <c r="H42" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5637,7 +6815,7 @@
         <v>3461</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C43" s="0" t="n">
         <v>42</v>
@@ -5652,10 +6830,10 @@
         <v>2844</v>
       </c>
       <c r="G43" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="H43" s="0" t="s">
         <v>96</v>
-      </c>
-      <c r="H43" s="0" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5663,7 +6841,7 @@
         <v>3461</v>
       </c>
       <c r="B44" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C44" s="0" t="n">
         <v>43</v>
@@ -5678,10 +6856,10 @@
         <v>2844</v>
       </c>
       <c r="G44" s="0" t="s">
-        <v>97</v>
+        <v>142</v>
       </c>
       <c r="H44" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5689,7 +6867,7 @@
         <v>3461</v>
       </c>
       <c r="B45" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C45" s="0" t="n">
         <v>44</v>
@@ -5704,10 +6882,10 @@
         <v>2844</v>
       </c>
       <c r="G45" s="0" t="s">
-        <v>98</v>
+        <v>143</v>
       </c>
       <c r="H45" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5715,25 +6893,25 @@
         <v>3461</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C46" s="0" t="n">
         <v>45</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>99</v>
+        <v>144</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="F46" s="0" t="n">
         <v>2844</v>
       </c>
       <c r="G46" s="0" t="s">
-        <v>101</v>
+        <v>146</v>
       </c>
       <c r="H46" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5741,13 +6919,13 @@
         <v>3461</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C47" s="0" t="n">
         <v>46</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>102</v>
+        <v>147</v>
       </c>
       <c r="E47" s="0" t="n">
         <v>570</v>
@@ -5756,10 +6934,10 @@
         <v>2844</v>
       </c>
       <c r="G47" s="0" t="s">
-        <v>103</v>
+        <v>148</v>
       </c>
       <c r="H47" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5767,13 +6945,13 @@
         <v>3461</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>78</v>
+        <v>123</v>
       </c>
       <c r="C48" s="0" t="n">
         <v>47</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>104</v>
+        <v>149</v>
       </c>
       <c r="E48" s="0" t="n">
         <v>406</v>
@@ -5782,10 +6960,10 @@
         <v>2844</v>
       </c>
       <c r="G48" s="0" t="s">
-        <v>105</v>
+        <v>150</v>
       </c>
       <c r="H48" s="0" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>